<commit_message>
Initial commit - Procurement System
</commit_message>
<xml_diff>
--- a/data/Design_boq.xlsx
+++ b/data/Design_boq.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Manisha\Desktop\ProcurementSystem\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B689C234-1306-464F-A4B1-028C2C1417FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C102C85-4993-495E-B3C8-2FDF7135E41F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="17">
   <si>
     <t>last_updated</t>
   </si>
@@ -40,9 +40,6 @@
   </si>
   <si>
     <t>xpx</t>
-  </si>
-  <si>
-    <t>unit</t>
   </si>
   <si>
     <t>remarks</t>
@@ -433,54 +430,50 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.109375" customWidth="1"/>
     <col min="2" max="2" width="14.21875" customWidth="1"/>
     <col min="3" max="3" width="15.77734375" customWidth="1"/>
     <col min="4" max="4" width="18.44140625" customWidth="1"/>
-    <col min="5" max="5" width="9" customWidth="1"/>
-    <col min="6" max="6" width="13.6640625" customWidth="1"/>
-    <col min="8" max="8" width="13" customWidth="1"/>
-    <col min="9" max="9" width="22" customWidth="1"/>
+    <col min="5" max="5" width="13.6640625" customWidth="1"/>
+    <col min="7" max="7" width="13" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="I1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="3" t="s">
+    </row>
+    <row r="2" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>15</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>4</v>
@@ -489,21 +482,20 @@
         <v>2</v>
       </c>
       <c r="D2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="1">
+        <v>15000</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" s="1">
-        <v>15000</v>
-      </c>
-      <c r="G2" s="1"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="1"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="G2" s="2"/>
+      <c r="H2" s="1"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>4</v>
@@ -512,90 +504,85 @@
         <v>3</v>
       </c>
       <c r="D3" s="1"/>
-      <c r="E3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F3" s="1">
+      <c r="E3" s="1">
         <v>120</v>
       </c>
-      <c r="G3" s="1"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="1"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="F3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G3" s="2"/>
+      <c r="H3" s="1"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>17</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="1">
+        <v>1500</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F4" s="1">
-        <v>1500</v>
-      </c>
-      <c r="H4" s="4"/>
-      <c r="I4" s="1"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="G4" s="4"/>
+      <c r="H4" s="1"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>17</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D5" s="1"/>
-      <c r="E5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F5" s="1">
+      <c r="E5" s="1">
         <v>12</v>
       </c>
-      <c r="H5" s="4"/>
-      <c r="I5" s="1"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="F5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="4"/>
+      <c r="H5" s="1"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
       <c r="C6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="I6" s="1"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H6" s="1"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="C7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="I7" s="1"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H7" s="1"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="C8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="I8" s="1"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H8" s="1"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="C9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="I9" s="1"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H9" s="1"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="C10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="I10" s="1"/>
+      <c r="H10" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix all 5 issues - login design, project id, vendor history, sidebar nav, page routing
</commit_message>
<xml_diff>
--- a/data/Design_boq.xlsx
+++ b/data/Design_boq.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Manisha\Desktop\ProcurementSystem\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C102C85-4993-495E-B3C8-2FDF7135E41F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EF5055C-0D26-4FC1-9043-D7B9EF74361A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="17">
   <si>
     <t>last_updated</t>
   </si>
@@ -556,7 +556,9 @@
       <c r="H5" s="1"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="1"/>
+      <c r="A6" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="C6" s="1"/>
       <c r="H6" s="1"/>
     </row>

</xml_diff>